<commit_message>
Changed endpoint values to be in centimeters (was inches). Small fix for the power curve.
</commit_message>
<xml_diff>
--- a/results/junipermarie_brachistochrone_points.xlsx
+++ b/results/junipermarie_brachistochrone_points.xlsx
@@ -445,399 +445,399 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>4.7</v>
+        <v>11.938</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.0001056719328906038</v>
+        <v>0.0002684067095421338</v>
       </c>
       <c r="B3" t="n">
-        <v>4.695094710516113</v>
+        <v>11.92554056471093</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.0008448461321486605</v>
+        <v>0.002145909175657598</v>
       </c>
       <c r="B4" t="n">
-        <v>4.680399317122591</v>
+        <v>11.88821426549138</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.002848380576627626</v>
+        <v>0.00723488666463417</v>
       </c>
       <c r="B5" t="n">
-        <v>4.655975159529375</v>
+        <v>11.82617690520461</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.00674185570761336</v>
+        <v>0.01712431349733793</v>
       </c>
       <c r="B6" t="n">
-        <v>4.621924186061509</v>
+        <v>11.73968743259623</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.01314296320762144</v>
+        <v>0.03338312654735847</v>
       </c>
       <c r="B7" t="n">
-        <v>4.578388528118935</v>
+        <v>11.62910686142209</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.02265892770748435</v>
+        <v>0.05755367637701025</v>
       </c>
       <c r="B8" t="n">
-        <v>4.525549906909025</v>
+        <v>11.49489676354892</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.03588397218372274</v>
+        <v>0.09114528934665576</v>
       </c>
       <c r="B9" t="n">
-        <v>4.463628874928192</v>
+        <v>11.33761734231761</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.05339683762582864</v>
+        <v>0.1356279675696048</v>
       </c>
       <c r="B10" t="n">
-        <v>4.392883895358688</v>
+        <v>11.15792509421107</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.07575836732656131</v>
+        <v>0.1924262530094658</v>
       </c>
       <c r="B11" t="n">
-        <v>4.313610263223271</v>
+        <v>10.95657006858711</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.1035091658786153</v>
+        <v>0.262913281331683</v>
       </c>
       <c r="B12" t="n">
-        <v>4.226138872800914</v>
+        <v>10.73439273691432</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.1371673426491899</v>
+        <v>0.3484050503289425</v>
       </c>
       <c r="B13" t="n">
-        <v>4.130834836448457</v>
+        <v>10.49232048457908</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.1772263491513705</v>
+        <v>0.4501549268444812</v>
       </c>
       <c r="B14" t="n">
-        <v>4.028095960593367</v>
+        <v>10.23136373990715</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.2241529193393038</v>
+        <v>0.5693484151218317</v>
       </c>
       <c r="B15" t="n">
-        <v>3.918351085258897</v>
+        <v>9.9526117565576</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.2783851214245331</v>
+        <v>0.7070982084183139</v>
       </c>
       <c r="B16" t="n">
-        <v>3.802058294052629</v>
+        <v>9.657228066893676</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.3403305293453605</v>
+        <v>0.8644395445372156</v>
       </c>
       <c r="B17" t="n">
-        <v>3.67970300209002</v>
+        <v>9.34644562530865</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.4103645215216701</v>
+        <v>1.042325884665042</v>
       </c>
       <c r="B18" t="n">
-        <v>3.551795929834126</v>
+        <v>9.02156166177868</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>0.4888287139963354</v>
+        <v>1.241624933550692</v>
       </c>
       <c r="B19" t="n">
-        <v>3.418870971308842</v>
+        <v>8.683932267124458</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0.576029534503405</v>
+        <v>1.463115017638649</v>
       </c>
       <c r="B20" t="n">
-        <v>3.281482965583903</v>
+        <v>8.334966732583112</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>0.6722369434150109</v>
+        <v>1.707481836274128</v>
       </c>
       <c r="B21" t="n">
-        <v>3.140205380833645</v>
+        <v>7.976121667317457</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>0.7776833069058741</v>
+        <v>1.97531559954092</v>
       </c>
       <c r="B22" t="n">
-        <v>2.995627920636439</v>
+        <v>7.608894918416555</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>0.8925624270388957</v>
+        <v>2.267108564678795</v>
       </c>
       <c r="B23" t="n">
-        <v>2.848354062506294</v>
+        <v>7.234819318765987</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>1.01702873282034</v>
+        <v>2.583252981363665</v>
       </c>
       <c r="B24" t="n">
-        <v>2.698998538930983</v>
+        <v>6.855456288884697</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>1.151196635601208</v>
+        <v>2.924039454427068</v>
       </c>
       <c r="B25" t="n">
-        <v>2.548184771431036</v>
+        <v>6.472389319434832</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1.295140051515391</v>
+        <v>3.289655730849093</v>
       </c>
       <c r="B26" t="n">
-        <v>2.396542268350043</v>
+        <v>6.087217361609111</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1.448892092948015</v>
+        <v>3.680185916087957</v>
       </c>
       <c r="B27" t="n">
-        <v>2.24470399723808</v>
+        <v>5.701548152984725</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>1.61244493032177</v>
+        <v>4.095610123017297</v>
       </c>
       <c r="B28" t="n">
-        <v>2.093303742796146</v>
+        <v>5.316991506702211</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1.785749824778182</v>
+        <v>4.535804554936583</v>
       </c>
       <c r="B29" t="n">
-        <v>1.942973461409737</v>
+        <v>4.935152591980732</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1.968717331617376</v>
+        <v>5.000542022308134</v>
       </c>
       <c r="B30" t="n">
-        <v>1.794340643313968</v>
+        <v>4.557625234017478</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>2.161217673647177</v>
+        <v>5.489492891063831</v>
       </c>
       <c r="B31" t="n">
-        <v>1.648025693400736</v>
+        <v>4.18598526123787</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>2.36308128288317</v>
+        <v>6.002226458523253</v>
       </c>
       <c r="B32" t="n">
-        <v>1.504639341600666</v>
+        <v>3.821783927665692</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>2.574099508338585</v>
+        <v>6.538212751180006</v>
       </c>
       <c r="B33" t="n">
-        <v>1.364780093649084</v>
+        <v>3.466541437868672</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>2.794025486949682</v>
+        <v>7.096824736852192</v>
       </c>
       <c r="B34" t="n">
-        <v>1.229031732876735</v>
+        <v>3.121740601506907</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3.022575174001287</v>
+        <v>7.677340941963268</v>
       </c>
       <c r="B35" t="n">
-        <v>1.097960883452963</v>
+        <v>2.788820643970526</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>3.25942852875143</v>
+        <v>8.27894846302863</v>
       </c>
       <c r="B36" t="n">
-        <v>0.972114645252542</v>
+        <v>2.469171198941456</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>3.50423085030619</v>
+        <v>8.900746359777722</v>
       </c>
       <c r="B37" t="n">
-        <v>0.85201831021844</v>
+        <v>2.164126507954839</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>3.756594258168681</v>
+        <v>9.541749415748448</v>
       </c>
       <c r="B38" t="n">
-        <v>0.7381731697525757</v>
+        <v>1.874959851171543</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>4.016099311282293</v>
+        <v>10.20089225065702</v>
       </c>
       <c r="B39" t="n">
-        <v>0.6310544222866854</v>
+        <v>1.602878232608182</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4.282296758810127</v>
+        <v>10.87703376737772</v>
       </c>
       <c r="B40" t="n">
-        <v>0.5311091897672782</v>
+        <v>1.349017342008885</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4.554709415342793</v>
+        <v>11.56896191497069</v>
       </c>
       <c r="B41" t="n">
-        <v>0.4387546513340004</v>
+        <v>1.114436814388361</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>4.83283415270724</v>
+        <v>12.27539874787639</v>
       </c>
       <c r="B42" t="n">
-        <v>0.3543763019816142</v>
+        <v>0.9001158070332984</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>5.116144000062724</v>
+        <v>12.99500576015932</v>
       </c>
       <c r="B43" t="n">
-        <v>0.2783263434740295</v>
+        <v>0.7069489124240356</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>5.404090343517896</v>
+        <v>13.72638947253546</v>
       </c>
       <c r="B44" t="n">
-        <v>0.2109222142268763</v>
+        <v>0.5357424241362665</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>5.696105216087663</v>
+        <v>14.46810724886266</v>
       </c>
       <c r="B45" t="n">
-        <v>0.1524452642949727</v>
+        <v>0.38721097130923</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>5.991603668431373</v>
+        <v>15.21867331781569</v>
       </c>
       <c r="B46" t="n">
-        <v>0.1031395809954114</v>
+        <v>0.2619745357283456</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>6.289986210476647</v>
+        <v>15.97656497461068</v>
       </c>
       <c r="B47" t="n">
-        <v>0.06321097006819976</v>
+        <v>0.1605558639732276</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>6.590641313737367</v>
+        <v>16.74022893689291</v>
       </c>
       <c r="B48" t="n">
-        <v>0.03282609662716052</v>
+        <v>0.0833782854329872</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>6.892947963880932</v>
+        <v>17.50808782825757</v>
       </c>
       <c r="B49" t="n">
-        <v>0.01211178948684477</v>
+        <v>0.03076394529658621</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>7.196278252890167</v>
+        <v>18.27854676234102</v>
       </c>
       <c r="B50" t="n">
-        <v>0.001154511769239974</v>
+        <v>0.002932459893870032</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>7.5</v>
+        <v>19.05</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>-1.77635683940025e-15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Had to change X-coordinate endpoint. Regenerated points for Junie-Marie and Marc's curves.
</commit_message>
<xml_diff>
--- a/results/junipermarie_brachistochrone_points.xlsx
+++ b/results/junipermarie_brachistochrone_points.xlsx
@@ -450,394 +450,394 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.0002684067095421338</v>
+        <v>0.0002559324108899195</v>
       </c>
       <c r="B3" t="n">
-        <v>11.92554056471093</v>
+        <v>11.92592955586505</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.002145909175657598</v>
+        <v>0.002046217306867668</v>
       </c>
       <c r="B4" t="n">
-        <v>11.88821426549138</v>
+        <v>11.88976703317904</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.00723488666463417</v>
+        <v>0.006899002652911144</v>
       </c>
       <c r="B5" t="n">
-        <v>11.82617690520461</v>
+        <v>11.82965866372468</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.01712431349733793</v>
+        <v>0.01633005246323478</v>
       </c>
       <c r="B6" t="n">
-        <v>11.73968743259623</v>
+        <v>11.74584751002553</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.03338312654735847</v>
+        <v>0.03183661744809348</v>
       </c>
       <c r="B7" t="n">
-        <v>11.62910686142209</v>
+        <v>11.63867248246474</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.05755367637701025</v>
+        <v>0.05489138052354578</v>
       </c>
       <c r="B8" t="n">
-        <v>11.49489676354892</v>
+        <v>11.50856696882002</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.09114528934665576</v>
+        <v>0.08693650166694969</v>
       </c>
       <c r="B9" t="n">
-        <v>11.33761734231761</v>
+        <v>11.35605708175694</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.1356279675696048</v>
+        <v>0.1293777861992391</v>
       </c>
       <c r="B10" t="n">
-        <v>11.15792509421107</v>
+        <v>11.18175953136685</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.1924262530094658</v>
+        <v>0.1835790000759223</v>
       </c>
       <c r="B11" t="n">
-        <v>10.95657006858711</v>
+        <v>10.98637913135262</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.262913281331683</v>
+        <v>0.2508563551742776</v>
       </c>
       <c r="B12" t="n">
-        <v>10.73439273691432</v>
+        <v>10.77070594894635</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.3484050503289425</v>
+        <v>0.3324731868768018</v>
       </c>
       <c r="B13" t="n">
-        <v>10.49232048457908</v>
+        <v>10.53561211008418</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.4501549268444812</v>
+        <v>0.4296348454733728</v>
       </c>
       <c r="B14" t="n">
-        <v>10.23136373990715</v>
+        <v>10.28204827275711</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.5693484151218317</v>
+        <v>0.5434838220399608</v>
       </c>
       <c r="B15" t="n">
-        <v>9.9526117565576</v>
+        <v>10.01103978279873</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.7070982084183139</v>
+        <v>0.6750951285035581</v>
       </c>
       <c r="B16" t="n">
-        <v>9.657228066893676</v>
+        <v>9.723682527654889</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.8644395445372156</v>
+        <v>0.8254719505751382</v>
       </c>
       <c r="B17" t="n">
-        <v>9.34644562530865</v>
+        <v>9.42113850490151</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>1.042325884665042</v>
+        <v>0.9955415911290385</v>
       </c>
       <c r="B18" t="n">
-        <v>9.02156166177868</v>
+        <v>9.104631123430334</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1.241624933550692</v>
+        <v>1.186151720432696</v>
       </c>
       <c r="B19" t="n">
-        <v>8.683932267124458</v>
+        <v>8.775440256303368</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1.463115017638649</v>
+        <v>1.398066948389805</v>
       </c>
       <c r="B20" t="n">
-        <v>8.334966732583112</v>
+        <v>8.434897065281</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1.707481836274128</v>
+        <v>1.631965732657873</v>
       </c>
       <c r="B21" t="n">
-        <v>7.976121667317457</v>
+        <v>8.084378617952027</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1.97531559954092</v>
+        <v>1.88843763514291</v>
       </c>
       <c r="B22" t="n">
-        <v>7.608894918416555</v>
+        <v>7.72530231923253</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2.267108564678795</v>
+        <v>2.167980937965293</v>
       </c>
       <c r="B23" t="n">
-        <v>7.234819318765987</v>
+        <v>7.359120179751139</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2.583252981363665</v>
+        <v>2.471000628537209</v>
       </c>
       <c r="B24" t="n">
-        <v>6.855456288884697</v>
+        <v>6.987312944297858</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2.924039454427068</v>
+        <v>2.797806761899497</v>
       </c>
       <c r="B25" t="n">
-        <v>6.472389319434832</v>
+        <v>6.611384104079442</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3.289655730849093</v>
+        <v>3.148613206940153</v>
       </c>
       <c r="B26" t="n">
-        <v>6.087217361609111</v>
+        <v>6.232853816994235</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3.680185916087957</v>
+        <v>3.523536781564493</v>
       </c>
       <c r="B27" t="n">
-        <v>5.701548152984725</v>
+        <v>5.853252760511253</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>4.095610123017297</v>
+        <v>3.922596780314107</v>
       </c>
       <c r="B28" t="n">
-        <v>5.316991506702211</v>
+        <v>5.474115942010867</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>4.535804554936583</v>
+        <v>4.345714896344766</v>
       </c>
       <c r="B29" t="n">
-        <v>4.935152591980732</v>
+        <v>5.096976491616488</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>5.000542022308134</v>
+        <v>4.792715538078833</v>
       </c>
       <c r="B30" t="n">
-        <v>4.557625234017478</v>
+        <v>4.723359462617347</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>5.489492891063831</v>
+        <v>5.263326539251659</v>
       </c>
       <c r="B31" t="n">
-        <v>4.18598526123787</v>
+        <v>4.35477566455192</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>6.002226458523253</v>
+        <v>5.757180259480777</v>
       </c>
       <c r="B32" t="n">
-        <v>3.821783927665692</v>
+        <v>3.992715553889317</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>6.538212751180006</v>
+        <v>6.273815070907439</v>
       </c>
       <c r="B33" t="n">
-        <v>3.466541437868672</v>
+        <v>3.6386432070132</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>7.096824736852192</v>
+        <v>6.812677224898938</v>
       </c>
       <c r="B34" t="n">
-        <v>3.121740601506907</v>
+        <v>3.293990399879815</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>7.677340941963268</v>
+        <v>7.373123091263218</v>
       </c>
       <c r="B35" t="n">
-        <v>2.788820643970526</v>
+        <v>2.960150818290575</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>8.27894846302863</v>
+        <v>7.954421760921041</v>
       </c>
       <c r="B36" t="n">
-        <v>2.469171198941456</v>
+        <v>2.638474422191184</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>8.900746359777722</v>
+        <v>8.555758001511089</v>
       </c>
       <c r="B37" t="n">
-        <v>2.164126507954839</v>
+        <v>2.33026198678675</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>9.541749415748448</v>
+        <v>9.176235553976424</v>
       </c>
       <c r="B38" t="n">
-        <v>1.874959851171543</v>
+        <v>2.036759842547095</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>10.20089225065702</v>
+        <v>9.814880756801664</v>
       </c>
       <c r="B39" t="n">
-        <v>1.602878232608182</v>
+        <v>1.759154835372323</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>10.87703376737772</v>
+        <v>10.47064648324548</v>
       </c>
       <c r="B40" t="n">
-        <v>1.349017342008885</v>
+        <v>1.498569527298462</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>11.56896191497069</v>
+        <v>11.14241637564721</v>
       </c>
       <c r="B41" t="n">
-        <v>1.114436814388361</v>
+        <v>1.25605765715021</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>12.27539874787639</v>
+        <v>11.82900935968529</v>
       </c>
       <c r="B42" t="n">
-        <v>0.9001158070332984</v>
+        <v>1.032599879496743</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>12.99500576015932</v>
+        <v>12.52918442033283</v>
       </c>
       <c r="B43" t="n">
-        <v>0.7069489124240356</v>
+        <v>0.8290997991411704</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>13.72638947253546</v>
+        <v>13.2416456201978</v>
       </c>
       <c r="B44" t="n">
-        <v>0.5357424241362665</v>
+        <v>0.6463803171790392</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>14.46810724886266</v>
+        <v>13.96504733995483</v>
       </c>
       <c r="B45" t="n">
-        <v>0.38721097130923</v>
+        <v>0.4851803034015738</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>15.21867331781569</v>
+        <v>14.69799971967783</v>
       </c>
       <c r="B46" t="n">
-        <v>0.2619745357283456</v>
+        <v>0.3461516084994898</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>15.97656497461068</v>
+        <v>15.43907427906998</v>
       </c>
       <c r="B47" t="n">
-        <v>0.1605558639732276</v>
+        <v>0.2298564281493114</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>16.74022893689291</v>
+        <v>16.18680969386437</v>
       </c>
       <c r="B48" t="n">
-        <v>0.0833782854329872</v>
+        <v>0.1367650296411078</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>17.50808782825757</v>
+        <v>16.93971770503711</v>
       </c>
       <c r="B49" t="n">
-        <v>0.03076394529658621</v>
+        <v>0.06725385024058106</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>18.27854676234102</v>
+        <v>17.6962891369376</v>
       </c>
       <c r="B50" t="n">
-        <v>0.002932459893870032</v>
+        <v>0.02160397497522482</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>19.05</v>
+        <v>18.455</v>
       </c>
       <c r="B51" t="n">
-        <v>-1.77635683940025e-15</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Endpoints changed (again) Chase added his wavy curve.
</commit_message>
<xml_diff>
--- a/results/junipermarie_brachistochrone_points.xlsx
+++ b/results/junipermarie_brachistochrone_points.xlsx
@@ -445,399 +445,399 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>11.938</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.0002559324108899195</v>
+        <v>0.006849455874539666</v>
       </c>
       <c r="B3" t="n">
-        <v>11.92592955586505</v>
+        <v>9.815068366171333</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.002046217306867668</v>
+        <v>0.05469433931276195</v>
       </c>
       <c r="B4" t="n">
-        <v>11.88976703317904</v>
+        <v>9.262552440402663</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.006899002652911144</v>
+        <v>0.1840248772157866</v>
       </c>
       <c r="B5" t="n">
-        <v>11.82965866372468</v>
+        <v>8.349261065249472</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.01633005246323478</v>
+        <v>0.4343271209199995</v>
       </c>
       <c r="B6" t="n">
-        <v>11.74584751002553</v>
+        <v>7.086449042411892</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.03183661744809348</v>
+        <v>0.8435963460935209</v>
       </c>
       <c r="B7" t="n">
-        <v>11.63867248246474</v>
+        <v>5.489678435967457</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.05489138052354578</v>
+        <v>1.447868823970637</v>
       </c>
       <c r="B8" t="n">
-        <v>11.50856696882002</v>
+        <v>3.578626795737686</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.08693650166694969</v>
+        <v>2.280777734067287</v>
       </c>
       <c r="B9" t="n">
-        <v>11.35605708175694</v>
+        <v>1.37684466411755</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.1293777861992391</v>
+        <v>3.373138691016996</v>
       </c>
       <c r="B10" t="n">
-        <v>11.18175953136685</v>
+        <v>-1.088534645305991</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.1835790000759223</v>
+        <v>4.752569993221601</v>
       </c>
       <c r="B11" t="n">
-        <v>10.98637913135262</v>
+        <v>-3.787129420849165</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>0.2508563551742776</v>
+        <v>6.443152273122511</v>
       </c>
       <c r="B12" t="n">
-        <v>10.77070594894635</v>
+        <v>-6.685683956946292</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0.3324731868768018</v>
+        <v>8.465131743338448</v>
       </c>
       <c r="B13" t="n">
-        <v>10.53561211008418</v>
+        <v>-9.748478375573409</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>0.4296348454733728</v>
+        <v>10.83467069566895</v>
       </c>
       <c r="B14" t="n">
-        <v>10.28204827275711</v>
+        <v>-12.93776881451113</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0.5434838220399608</v>
+        <v>13.56364832764963</v>
       </c>
       <c r="B15" t="n">
-        <v>10.01103978279873</v>
+        <v>-16.21425255785636</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0.6750951285035581</v>
+        <v>16.65951435114167</v>
       </c>
       <c r="B16" t="n">
-        <v>9.723682527654889</v>
+        <v>-19.53755237682064</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>0.8254719505751382</v>
+        <v>20.12519718698688</v>
       </c>
       <c r="B17" t="n">
-        <v>9.42113850490151</v>
+        <v>-22.866714112118</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0.9955415911290385</v>
+        <v>23.95906787707701</v>
       </c>
       <c r="B18" t="n">
-        <v>9.104631123430334</v>
+        <v>-26.16071136606435</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1.186151720432696</v>
+        <v>28.15496015856113</v>
       </c>
       <c r="B19" t="n">
-        <v>8.775440256303368</v>
+        <v>-29.37895108489553</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>1.398066948389805</v>
+        <v>32.70224645280983</v>
       </c>
       <c r="B20" t="n">
-        <v>8.434897065281</v>
+        <v>-32.48177380083993</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1.631965732657873</v>
+        <v>37.58596883269828</v>
       </c>
       <c r="B21" t="n">
-        <v>8.084378617952027</v>
+        <v>-35.4309423692921</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1.88843763514291</v>
+        <v>42.78702335425353</v>
       </c>
       <c r="B22" t="n">
-        <v>7.72530231923253</v>
+        <v>-38.1901131782119</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2.167980937965293</v>
+        <v>48.28239548108412</v>
       </c>
       <c r="B23" t="n">
-        <v>7.359120179751139</v>
+        <v>-40.72528402287466</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>2.471000628537209</v>
+        <v>54.04544370037643</v>
       </c>
       <c r="B24" t="n">
-        <v>6.987312944297858</v>
+        <v>-43.00521312665913</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>2.797806761899497</v>
+        <v>60.04622783536092</v>
       </c>
       <c r="B25" t="n">
-        <v>6.611384104079442</v>
+        <v>-45.0018041441365</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>3.148613206940153</v>
+        <v>66.25187800834131</v>
       </c>
       <c r="B26" t="n">
-        <v>6.232853816994235</v>
+        <v>-46.690452401936</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>3.523536781564493</v>
+        <v>72.62699970742959</v>
       </c>
       <c r="B27" t="n">
-        <v>5.853252760511253</v>
+        <v>-48.05034811054261</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>3.922596780314107</v>
+        <v>79.13410996521081</v>
       </c>
       <c r="B28" t="n">
-        <v>5.474115942010867</v>
+        <v>-49.06473281044426</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>4.345714896344766</v>
+        <v>85.73409927415891</v>
       </c>
       <c r="B29" t="n">
-        <v>5.096976491616488</v>
+        <v>-49.72110589235494</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4.792715538078833</v>
+        <v>92.38671354646233</v>
       </c>
       <c r="B30" t="n">
-        <v>4.723359462617347</v>
+        <v>-50.01137864649466</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>5.263326539251659</v>
+        <v>99.05105017890335</v>
       </c>
       <c r="B31" t="n">
-        <v>4.35477566455192</v>
+        <v>-49.93197394252398</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>5.757180259480777</v>
+        <v>105.6860621096146</v>
       </c>
       <c r="B32" t="n">
-        <v>3.992715553889317</v>
+        <v>-49.4838703117436</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>6.273815070907439</v>
+        <v>112.2510636550488</v>
       </c>
       <c r="B33" t="n">
-        <v>3.6386432070132</v>
+        <v>-48.67258988831875</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>6.812677224898938</v>
+        <v>118.70623189356</v>
       </c>
       <c r="B34" t="n">
-        <v>3.293990399879815</v>
+        <v>-47.5081303581329</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>7.373123091263218</v>
+        <v>125.0130974168748</v>
       </c>
       <c r="B35" t="n">
-        <v>2.960150818290575</v>
+        <v>-46.00484175388822</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>7.954421760921041</v>
+        <v>131.1350184017564</v>
       </c>
       <c r="B36" t="n">
-        <v>2.638474422191184</v>
+        <v>-44.18124961474907</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>8.555758001511089</v>
+        <v>137.0376321597132</v>
       </c>
       <c r="B37" t="n">
-        <v>2.33026198678675</v>
+        <v>-42.05982668979237</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>9.176235553976424</v>
+        <v>142.6892786001512</v>
       </c>
       <c r="B38" t="n">
-        <v>2.036759842547095</v>
+        <v>-39.66671599864151</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>9.814880756801664</v>
+        <v>148.0613903884891</v>
       </c>
       <c r="B39" t="n">
-        <v>1.759154835372323</v>
+        <v>-37.03140866210213</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>10.47064648324548</v>
+        <v>153.1288449911843</v>
       </c>
       <c r="B40" t="n">
-        <v>1.498569527298462</v>
+        <v>-34.18638047300291</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>11.14241637564721</v>
+        <v>157.8702742692984</v>
       </c>
       <c r="B41" t="n">
-        <v>1.25605765715021</v>
+        <v>-31.166691685903</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>11.82900935968529</v>
+        <v>162.2683278053751</v>
       </c>
       <c r="B42" t="n">
-        <v>1.032599879496743</v>
+        <v>-28.00955495759479</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>12.52918442033283</v>
+        <v>166.3098867185634</v>
       </c>
       <c r="B43" t="n">
-        <v>0.8290997991411704</v>
+        <v>-24.75387676281787</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>13.2416456201978</v>
+        <v>169.9862253330691</v>
       </c>
       <c r="B44" t="n">
-        <v>0.6463803171790392</v>
+        <v>-21.43977793647613</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>13.96504733995483</v>
+        <v>173.2931187076398</v>
       </c>
       <c r="B45" t="n">
-        <v>0.4851803034015738</v>
+        <v>-18.10809925087942</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>14.69799971967783</v>
+        <v>176.2308947009588</v>
       </c>
       <c r="B46" t="n">
-        <v>0.3461516084994898</v>
+        <v>-14.79989812095038</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>15.43907427906998</v>
+        <v>178.8044299313314</v>
       </c>
       <c r="B47" t="n">
-        <v>0.2298564281493114</v>
+        <v>-11.55594263967059</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>16.18680969386437</v>
+        <v>181.0230896804505</v>
       </c>
       <c r="B48" t="n">
-        <v>0.1367650296411078</v>
+        <v>-8.416209178939745</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>16.93971770503711</v>
+        <v>182.9006124818305</v>
       </c>
       <c r="B49" t="n">
-        <v>0.06725385024058106</v>
+        <v>-5.419389747084161</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>17.6962891369376</v>
+        <v>184.4549408161638</v>
       </c>
       <c r="B50" t="n">
-        <v>0.02160397497522482</v>
+        <v>-2.602415174016731</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>18.455</v>
+        <v>185.708</v>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>5.329070518200751e-15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>